<commit_message>
Grand Total added in both sheets of Workbook #3
</commit_message>
<xml_diff>
--- a/Soldering Tools Required.xlsx
+++ b/Soldering Tools Required.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Electronics-DemandSystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XPENDER\Documents\GitHub\Electronics-DemandSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADDFD19-8647-4FFA-8EB3-AAD782DF842D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="International Supplier" sheetId="1" r:id="rId1"/>
     <sheet name="Local Supplier" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="67">
   <si>
     <t>Manufacturer</t>
   </si>
@@ -52,18 +51,6 @@
   </si>
   <si>
     <t>Link</t>
-  </si>
-  <si>
-    <t>LE-UVWE5D</t>
-  </si>
-  <si>
-    <t>Magnifying LED lamp 2.25X (5-Diopter Lens), ESD safe. UV (400 nm) + White LEDs (1100 lm)</t>
-  </si>
-  <si>
-    <t>Ideal Tek</t>
-  </si>
-  <si>
-    <t>Ideal-Tek</t>
   </si>
   <si>
     <t>PANAVISE 350 Multi-Purpose Work Center</t>
@@ -199,9 +186,6 @@
     <t>Magnifying Glass</t>
   </si>
   <si>
-    <t>Need Quotation from Manufacturer or search some of it's distributor</t>
-  </si>
-  <si>
     <t>PANAVISE 350</t>
   </si>
   <si>
@@ -245,18 +229,24 @@
   </si>
   <si>
     <t>TOMLOV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grand Total </t>
+  </si>
+  <si>
+    <t>Grand Total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$PKR]\ #,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,6 +286,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -437,7 +435,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -483,31 +481,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -525,19 +526,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -854,8 +862,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K40"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
@@ -872,127 +880,129 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
+      <c r="A1" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="25" t="s">
+      <c r="B3" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="25" t="s">
+      <c r="F3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="J3" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="K3" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
+      <c r="H3" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="K3" s="21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="9">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" s="20" t="s">
+      <c r="B4" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="20"/>
-      <c r="G4" s="22" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23">
-        <f>H4+I4</f>
-        <v>0</v>
-      </c>
-      <c r="K4" s="21" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="9"/>
+      <c r="G4" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="12">
+        <v>100</v>
+      </c>
+      <c r="I4" s="12">
+        <v>74</v>
+      </c>
+      <c r="J4" s="19">
+        <f t="shared" ref="J4:J9" si="0">H4+I4</f>
+        <v>174</v>
+      </c>
+      <c r="K4" s="13"/>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F5" s="9"/>
       <c r="G5" s="11" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="H5" s="12">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="I5" s="12">
-        <v>74</v>
-      </c>
-      <c r="J5" s="23">
-        <f t="shared" ref="J5:J10" si="0">H5+I5</f>
-        <v>174</v>
+        <v>3</v>
+      </c>
+      <c r="J5" s="19">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="K5" s="13"/>
     </row>
@@ -1001,154 +1011,133 @@
         <v>3</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H6" s="12">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I6" s="12">
-        <v>3</v>
-      </c>
-      <c r="J6" s="23">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="K6" s="13"/>
-    </row>
-    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="9">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="12">
-        <v>6</v>
-      </c>
-      <c r="I7" s="12">
-        <v>4</v>
-      </c>
-      <c r="J7" s="23">
+      <c r="J6" s="19">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="K7" s="13"/>
-    </row>
-    <row r="8" spans="1:11" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="31">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" s="31"/>
-      <c r="D8" s="32" t="s">
-        <v>63</v>
-      </c>
-      <c r="E8" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="F8" s="31"/>
-      <c r="G8" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" s="34">
+      <c r="K6" s="13"/>
+    </row>
+    <row r="7" spans="1:11" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="22">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="22"/>
+      <c r="D7" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="22"/>
+      <c r="G7" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="25">
         <v>6.07</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I7" s="25">
         <v>5.35</v>
       </c>
-      <c r="J8" s="35">
+      <c r="J7" s="26">
         <f t="shared" si="0"/>
         <v>11.42</v>
       </c>
-      <c r="K8" s="31"/>
+      <c r="K7" s="22"/>
+    </row>
+    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="9">
+        <v>5</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F8" s="9"/>
+      <c r="G8" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="12">
+        <v>28.08</v>
+      </c>
+      <c r="I8" s="12">
+        <v>1.05</v>
+      </c>
+      <c r="J8" s="12">
+        <f t="shared" si="0"/>
+        <v>29.13</v>
+      </c>
+      <c r="K8" s="13"/>
     </row>
     <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H9" s="12">
-        <v>28.08</v>
+        <v>155.22</v>
       </c>
       <c r="I9" s="12">
-        <v>1.05</v>
+        <v>41.62</v>
       </c>
       <c r="J9" s="12">
         <f t="shared" si="0"/>
-        <v>29.13</v>
+        <v>196.84</v>
       </c>
       <c r="K9" s="13"/>
     </row>
-    <row r="10" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" s="9">
-        <v>7</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="12">
-        <v>155.22</v>
-      </c>
-      <c r="I10" s="12">
-        <v>41.62</v>
-      </c>
-      <c r="J10" s="12">
-        <f t="shared" si="0"/>
-        <v>196.84</v>
-      </c>
-      <c r="K10" s="13"/>
+    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B10" s="4"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="J10" s="32">
+        <f>SUM(J4:J9)</f>
+        <v>426.39</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B11" s="4"/>
@@ -1157,7 +1146,6 @@
       <c r="J11" s="7"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="4"/>
       <c r="H12" s="6"/>
       <c r="I12" s="7"/>
       <c r="J12" s="7"/>
@@ -1234,8 +1222,6 @@
     </row>
     <row r="27" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H27" s="6"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
     </row>
     <row r="28" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H28" s="6"/>
@@ -1259,7 +1245,7 @@
       <c r="H34" s="6"/>
     </row>
     <row r="35" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H35" s="6"/>
+      <c r="H35" s="5"/>
     </row>
     <row r="36" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H36" s="5"/>
@@ -1272,31 +1258,26 @@
     </row>
     <row r="39" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H39" s="5"/>
-    </row>
-    <row r="40" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H40" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:K2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="G5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="G6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="G7" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="G8" r:id="rId5" xr:uid="{081964B0-AEAA-4DF3-988B-629FF5C89D75}"/>
-    <hyperlink ref="G9" r:id="rId6" xr:uid="{7D5B5EEC-5F43-48FB-92F3-22FD8C82C72B}"/>
-    <hyperlink ref="G10" r:id="rId7" xr:uid="{00442A6D-4CEE-43D8-915A-1E57D1B16373}"/>
+    <hyperlink ref="G5" r:id="rId1"/>
+    <hyperlink ref="G6" r:id="rId2"/>
+    <hyperlink ref="G7" r:id="rId3"/>
+    <hyperlink ref="G8" r:id="rId4"/>
+    <hyperlink ref="G9" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId8"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J40"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" style="3" bestFit="1" customWidth="1"/>
@@ -1304,44 +1285,44 @@
     <col min="3" max="3" width="28.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10" style="4" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" style="4" customWidth="1"/>
     <col min="9" max="9" width="40.28515625" customWidth="1"/>
     <col min="10" max="10" width="19.28515625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30"/>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-    </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="31"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1</v>
@@ -1359,250 +1340,266 @@
         <v>5</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>1</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>15</v>
-      </c>
       <c r="G4" s="11" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H4" s="14">
         <v>1200</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J4" s="9"/>
     </row>
-    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H5" s="14">
         <v>750</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J5" s="9"/>
     </row>
-    <row r="6" spans="1:10" s="18" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" s="17" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>3</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H6" s="14">
         <v>1200</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J6" s="9"/>
     </row>
-    <row r="7" spans="1:10" s="18" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" s="17" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>4</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H7" s="14">
         <v>1800</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="1:10" s="18" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" s="17" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>5</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H8" s="14">
         <v>1580</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J8" s="9"/>
     </row>
-    <row r="9" spans="1:10" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>34</v>
+        <v>29</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>30</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H9" s="14">
         <v>1550</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J9" s="9"/>
     </row>
-    <row r="10" spans="1:10" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="17" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>7</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H10" s="14">
         <v>1750</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J10" s="9"/>
     </row>
-    <row r="11" spans="1:10" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="H12" s="8"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" s="17" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="33"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" s="39">
+        <f>SUM(H4:H10)</f>
+        <v>9830</v>
+      </c>
+      <c r="I11" s="33"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="34"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="36"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="37"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H13" s="8"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H14" s="8"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H15" s="8"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H16" s="8"/>
     </row>
     <row r="17" spans="8:8" x14ac:dyDescent="0.25">
@@ -1682,13 +1679,13 @@
     <mergeCell ref="A1:J2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="G6" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="G7" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="G8" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
-    <hyperlink ref="G9" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
-    <hyperlink ref="G10" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
-    <hyperlink ref="G5" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
+    <hyperlink ref="G4" r:id="rId1"/>
+    <hyperlink ref="G6" r:id="rId2"/>
+    <hyperlink ref="G7" r:id="rId3"/>
+    <hyperlink ref="G8" r:id="rId4"/>
+    <hyperlink ref="G9" r:id="rId5"/>
+    <hyperlink ref="G10" r:id="rId6"/>
+    <hyperlink ref="G5" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId8"/>

</xml_diff>

<commit_message>
VISE Link updated in sheet.
</commit_message>
<xml_diff>
--- a/Soldering Tools Required.xlsx
+++ b/Soldering Tools Required.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XPENDER\Documents\GitHub\Electronics-DemandSystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\Electronics-DemandSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="International Supplier" sheetId="1" r:id="rId1"/>
     <sheet name="Local Supplier" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -240,7 +240,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -511,6 +511,28 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -525,28 +547,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -880,32 +880,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="29"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
+      <c r="A2" s="37"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
@@ -1131,10 +1131,10 @@
     <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
       <c r="H10" s="6"/>
-      <c r="I10" s="32" t="s">
+      <c r="I10" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="J10" s="32">
+      <c r="J10" s="27">
         <f>SUM(J4:J9)</f>
         <v>426.39</v>
       </c>
@@ -1269,9 +1269,10 @@
     <hyperlink ref="G7" r:id="rId3"/>
     <hyperlink ref="G8" r:id="rId4"/>
     <hyperlink ref="G9" r:id="rId5"/>
+    <hyperlink ref="G4" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 
@@ -1292,30 +1293,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31"/>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
+      <c r="A2" s="39"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1560,35 +1561,35 @@
       <c r="J10" s="9"/>
     </row>
     <row r="11" spans="1:11" s="17" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="33"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="38" t="s">
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="H11" s="39">
+      <c r="H11" s="34">
         <f>SUM(H4:H10)</f>
         <v>9830</v>
       </c>
-      <c r="I11" s="33"/>
-      <c r="J11" s="33"/>
-      <c r="K11" s="34"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="29"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="36"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="37"/>
-      <c r="J12" s="33"/>
-      <c r="K12" s="37"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="32"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H13" s="8"/>

</xml_diff>

<commit_message>
#3 Exel File Links Completed
</commit_message>
<xml_diff>
--- a/Soldering Tools Required.xlsx
+++ b/Soldering Tools Required.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\Electronics-DemandSystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Electronics-DemandSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A83FA8-D795-4E15-9F10-EC4DBC5E9142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="International Supplier" sheetId="1" r:id="rId1"/>
     <sheet name="Local Supplier" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="86">
   <si>
     <t>Manufacturer</t>
   </si>
@@ -262,12 +263,42 @@
   </si>
   <si>
     <t>KADA</t>
+  </si>
+  <si>
+    <t>Hallroad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 Gram Solder Wire </t>
+  </si>
+  <si>
+    <t>Fine</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> BON-102</t>
+  </si>
+  <si>
+    <t>Flux Coating Tool Pen BONPEN BONKOTE</t>
+  </si>
+  <si>
+    <t>BONKOTE</t>
+  </si>
+  <si>
+    <t>Test Instrument</t>
+  </si>
+  <si>
+    <t>Daraz</t>
+  </si>
+  <si>
+    <t>Silicone Glue Sticks</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -462,7 +493,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -541,19 +572,12 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -568,12 +592,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -889,7 +907,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -907,32 +925,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="35"/>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
+      <c r="A2" s="32"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
@@ -1291,12 +1309,12 @@
     <mergeCell ref="A1:K2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G5" r:id="rId1"/>
-    <hyperlink ref="G6" r:id="rId2"/>
-    <hyperlink ref="G7" r:id="rId3"/>
-    <hyperlink ref="G8" r:id="rId4"/>
-    <hyperlink ref="G9" r:id="rId5"/>
-    <hyperlink ref="G4" r:id="rId6"/>
+    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="G6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="G7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="G8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="G9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="G4" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId7"/>
@@ -1304,8 +1322,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L44"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" style="3" bestFit="1" customWidth="1"/>
@@ -1313,41 +1331,42 @@
     <col min="3" max="3" width="28.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="13.85546875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" style="4" customWidth="1"/>
     <col min="9" max="9" width="17.28515625" style="4" customWidth="1"/>
     <col min="10" max="10" width="40.28515625" customWidth="1"/>
     <col min="11" max="11" width="19.28515625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-    </row>
-    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-    </row>
-    <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="34"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -1382,7 +1401,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -1415,7 +1434,7 @@
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2</v>
       </c>
@@ -1448,7 +1467,7 @@
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" spans="1:12" s="17" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" s="17" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>3</v>
       </c>
@@ -1481,7 +1500,7 @@
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:12" s="17" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" s="17" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>4</v>
       </c>
@@ -1514,7 +1533,7 @@
       </c>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" spans="1:12" s="17" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" s="17" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>5</v>
       </c>
@@ -1547,7 +1566,7 @@
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:12" s="17" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>6</v>
       </c>
@@ -1580,7 +1599,7 @@
       </c>
       <c r="K9" s="9"/>
     </row>
-    <row r="10" spans="1:12" s="17" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="17" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>7</v>
       </c>
@@ -1613,7 +1632,7 @@
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:12" s="17" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>8</v>
       </c>
@@ -1621,33 +1640,63 @@
         <v>67</v>
       </c>
       <c r="C11" s="9"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="9"/>
+      <c r="D11" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="H11" s="11">
+        <v>4</v>
+      </c>
+      <c r="I11" s="14">
+        <v>450</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>57</v>
+      </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" spans="1:12" s="17" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" s="17" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
         <v>9</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="9"/>
+      <c r="C12" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="H12" s="11">
+        <v>2</v>
+      </c>
+      <c r="I12" s="14">
+        <v>650</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>57</v>
+      </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:12" s="17" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
       <c r="B13" s="9" t="s">
         <v>70</v>
@@ -1673,60 +1722,61 @@
       <c r="I13" s="14">
         <v>6500</v>
       </c>
-      <c r="J13" s="9"/>
+      <c r="J13" s="9" t="s">
+        <v>57</v>
+      </c>
       <c r="K13" s="9"/>
     </row>
-    <row r="14" spans="1:12" s="17" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
         <v>10</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="11"/>
+      <c r="C14" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>83</v>
+      </c>
       <c r="H14" s="11">
-        <v>20</v>
-      </c>
-      <c r="I14" s="14"/>
-      <c r="J14" s="9"/>
+        <v>36</v>
+      </c>
+      <c r="I14" s="14">
+        <v>936</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>57</v>
+      </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:12" s="17" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="28"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="38" t="s">
+    <row r="15" spans="1:11" s="17" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="G15" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="H15" s="38"/>
-      <c r="I15" s="39">
-        <f>SUM(I4:I10)</f>
-        <v>9830</v>
-      </c>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
-      <c r="L15" s="29"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="31"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="28"/>
-      <c r="L16" s="32"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="29">
+        <f>SUM(I4:I14)</f>
+        <v>18366</v>
+      </c>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I16" s="8"/>
     </row>
     <row r="17" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I17" s="8"/>
@@ -1817,16 +1867,19 @@
     <mergeCell ref="A1:K2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1"/>
-    <hyperlink ref="G6" r:id="rId2"/>
-    <hyperlink ref="G7" r:id="rId3"/>
-    <hyperlink ref="G8" r:id="rId4"/>
-    <hyperlink ref="G9" r:id="rId5"/>
-    <hyperlink ref="G10" r:id="rId6"/>
-    <hyperlink ref="G5" r:id="rId7"/>
-    <hyperlink ref="G13" r:id="rId8"/>
+    <hyperlink ref="G4" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="G6" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="G7" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="G8" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="G9" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="G10" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+    <hyperlink ref="G5" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
+    <hyperlink ref="G13" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
+    <hyperlink ref="G11" r:id="rId9" xr:uid="{DD2885EE-EE98-4E6E-AF08-9025BACBF128}"/>
+    <hyperlink ref="G12" r:id="rId10" xr:uid="{75C4C36D-0A00-48A7-B29B-3AF497CC9A6A}"/>
+    <hyperlink ref="G14" r:id="rId11" xr:uid="{2BCD4C86-5E3F-4670-8813-371CA87A7CDF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId9"/>
+  <pageSetup orientation="portrait" r:id="rId12"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Equipment added to local suppler section
</commit_message>
<xml_diff>
--- a/Soldering Tools Required.xlsx
+++ b/Soldering Tools Required.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Electronics-DemandSystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A83FA8-D795-4E15-9F10-EC4DBC5E9142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="International Supplier" sheetId="1" r:id="rId1"/>
     <sheet name="Local Supplier" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="101">
   <si>
     <t>Manufacturer</t>
   </si>
@@ -293,12 +292,57 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>AliE</t>
+  </si>
+  <si>
+    <t>TOMLOV DM202</t>
+  </si>
+  <si>
+    <t>With customs</t>
+  </si>
+  <si>
+    <t>Solder Paste</t>
+  </si>
+  <si>
+    <t>Solder Wick</t>
+  </si>
+  <si>
+    <t>Heat Sink paste</t>
+  </si>
+  <si>
+    <t>Desolder Pump (small)</t>
+  </si>
+  <si>
+    <t>2 in 1 (Hot air / Soldering Iron)</t>
+  </si>
+  <si>
+    <t>Power Supply</t>
+  </si>
+  <si>
+    <t>Tablet Oscilloscope</t>
+  </si>
+  <si>
+    <t>Optional</t>
+  </si>
+  <si>
+    <t>Handheld Oscilloscope</t>
+  </si>
+  <si>
+    <t>DMM</t>
+  </si>
+  <si>
+    <t>With light</t>
+  </si>
+  <si>
+    <t>Market survey</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -493,7 +537,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -576,6 +620,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -907,7 +963,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -925,32 +981,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="32"/>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
+      <c r="A2" s="36"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
@@ -1309,12 +1365,12 @@
     <mergeCell ref="A1:K2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="G6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="G7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="G8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="G9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="G4" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="G5" r:id="rId1"/>
+    <hyperlink ref="G6" r:id="rId2"/>
+    <hyperlink ref="G7" r:id="rId3"/>
+    <hyperlink ref="G8" r:id="rId4"/>
+    <hyperlink ref="G9" r:id="rId5"/>
+    <hyperlink ref="G4" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId7"/>
@@ -1322,49 +1378,49 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K44"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.85546875" style="4" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="40.28515625" customWidth="1"/>
     <col min="11" max="11" width="19.28515625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
+      <c r="A2" s="38"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1725,7 +1781,9 @@
       <c r="J13" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="K13" s="9"/>
+      <c r="K13" s="9" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="14" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
@@ -1760,70 +1818,250 @@
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" s="17" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="G15" s="28" t="s">
+    <row r="15" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="30">
+        <v>11</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="31"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="H15" s="32"/>
+      <c r="I15" s="33">
+        <v>50000</v>
+      </c>
+      <c r="J15" s="30"/>
+      <c r="K15" s="30" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="30"/>
+      <c r="B16" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" s="30"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="32"/>
+      <c r="I16" s="33">
+        <v>800</v>
+      </c>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
+    </row>
+    <row r="17" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="30"/>
+      <c r="B17" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="30"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="32"/>
+      <c r="I17" s="33">
+        <v>500</v>
+      </c>
+      <c r="J17" s="30"/>
+      <c r="K17" s="30"/>
+    </row>
+    <row r="18" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="30"/>
+      <c r="B18" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" s="30"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" s="32"/>
+      <c r="I18" s="33">
+        <v>800</v>
+      </c>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+    </row>
+    <row r="19" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="30"/>
+      <c r="B19" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" s="30"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" s="32"/>
+      <c r="I19" s="33">
+        <v>500</v>
+      </c>
+      <c r="J19" s="30"/>
+      <c r="K19" s="30"/>
+    </row>
+    <row r="20" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="30"/>
+      <c r="B20" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="C20" s="30"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" s="32"/>
+      <c r="I20" s="33">
+        <v>36000</v>
+      </c>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="30"/>
+      <c r="B21" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="30"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H21" s="32">
+        <v>2</v>
+      </c>
+      <c r="I21" s="33">
+        <v>19500</v>
+      </c>
+      <c r="J21" s="30"/>
+      <c r="K21" s="30"/>
+    </row>
+    <row r="22" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="30"/>
+      <c r="B22" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="30"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" s="32">
+        <v>1</v>
+      </c>
+      <c r="I22" s="33">
+        <v>31000</v>
+      </c>
+      <c r="J22" s="30"/>
+      <c r="K22" s="30" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="30"/>
+      <c r="B23" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" s="30"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" s="32">
+        <v>1</v>
+      </c>
+      <c r="I23" s="33">
+        <v>20500</v>
+      </c>
+      <c r="J23" s="30"/>
+      <c r="K23" s="30"/>
+    </row>
+    <row r="24" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="30"/>
+      <c r="B24" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" s="30"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="H24" s="32">
+        <v>2</v>
+      </c>
+      <c r="I24" s="33">
+        <v>40000</v>
+      </c>
+      <c r="J24" s="30"/>
+      <c r="K24" s="30" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" s="17" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="G25" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="H15" s="28"/>
-      <c r="I15" s="29">
-        <f>SUM(I4:I14)</f>
-        <v>18366</v>
-      </c>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I16" s="8"/>
-    </row>
-    <row r="17" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I17" s="8"/>
-    </row>
-    <row r="18" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I18" s="8"/>
-    </row>
-    <row r="19" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I19" s="8"/>
-    </row>
-    <row r="20" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I20" s="8"/>
-    </row>
-    <row r="21" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I21" s="8"/>
-    </row>
-    <row r="22" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I22" s="8"/>
-    </row>
-    <row r="23" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I23" s="8"/>
-    </row>
-    <row r="24" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I24" s="8"/>
-    </row>
-    <row r="25" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I25" s="8"/>
-    </row>
-    <row r="26" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="H25" s="28"/>
+      <c r="I25" s="29">
+        <f>SUM(I4:I24)</f>
+        <v>217966</v>
+      </c>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I26" s="8"/>
     </row>
-    <row r="27" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I27" s="8"/>
     </row>
-    <row r="28" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I28" s="8"/>
     </row>
-    <row r="29" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I29" s="8"/>
     </row>
-    <row r="30" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I30" s="8"/>
     </row>
-    <row r="31" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I31" s="8"/>
     </row>
-    <row r="32" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I32" s="8"/>
     </row>
     <row r="33" spans="9:9" x14ac:dyDescent="0.25">
@@ -1839,47 +2077,86 @@
       <c r="I36" s="8"/>
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I37" s="5"/>
+      <c r="I37" s="8"/>
     </row>
     <row r="38" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I38" s="5"/>
+      <c r="I38" s="8"/>
     </row>
     <row r="39" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I39" s="5"/>
+      <c r="I39" s="8"/>
     </row>
     <row r="40" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I40" s="5"/>
+      <c r="I40" s="8"/>
     </row>
     <row r="41" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I41" s="5"/>
+      <c r="I41" s="8"/>
     </row>
     <row r="42" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I42" s="5"/>
+      <c r="I42" s="8"/>
     </row>
     <row r="43" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I43" s="5"/>
+      <c r="I43" s="8"/>
     </row>
     <row r="44" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I44" s="5"/>
+      <c r="I44" s="8"/>
+    </row>
+    <row r="45" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I45" s="8"/>
+    </row>
+    <row r="46" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I46" s="8"/>
+    </row>
+    <row r="47" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I47" s="5"/>
+    </row>
+    <row r="48" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I48" s="5"/>
+    </row>
+    <row r="49" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I49" s="5"/>
+    </row>
+    <row r="50" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I50" s="5"/>
+    </row>
+    <row r="51" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I51" s="5"/>
+    </row>
+    <row r="52" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I52" s="5"/>
+    </row>
+    <row r="53" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I53" s="5"/>
+    </row>
+    <row r="54" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I54" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:K2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="G6" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="G7" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="G8" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
-    <hyperlink ref="G9" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
-    <hyperlink ref="G10" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
-    <hyperlink ref="G5" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
-    <hyperlink ref="G13" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
-    <hyperlink ref="G11" r:id="rId9" xr:uid="{DD2885EE-EE98-4E6E-AF08-9025BACBF128}"/>
-    <hyperlink ref="G12" r:id="rId10" xr:uid="{75C4C36D-0A00-48A7-B29B-3AF497CC9A6A}"/>
-    <hyperlink ref="G14" r:id="rId11" xr:uid="{2BCD4C86-5E3F-4670-8813-371CA87A7CDF}"/>
+    <hyperlink ref="G4" r:id="rId1"/>
+    <hyperlink ref="G6" r:id="rId2"/>
+    <hyperlink ref="G7" r:id="rId3"/>
+    <hyperlink ref="G8" r:id="rId4"/>
+    <hyperlink ref="G9" r:id="rId5"/>
+    <hyperlink ref="G10" r:id="rId6"/>
+    <hyperlink ref="G5" r:id="rId7"/>
+    <hyperlink ref="G13" r:id="rId8"/>
+    <hyperlink ref="G11" r:id="rId9"/>
+    <hyperlink ref="G12" r:id="rId10"/>
+    <hyperlink ref="G14" r:id="rId11"/>
+    <hyperlink ref="G15" r:id="rId12"/>
+    <hyperlink ref="G16" r:id="rId13"/>
+    <hyperlink ref="G17" r:id="rId14"/>
+    <hyperlink ref="G18" r:id="rId15"/>
+    <hyperlink ref="G19" r:id="rId16"/>
+    <hyperlink ref="G20" r:id="rId17"/>
+    <hyperlink ref="G21" r:id="rId18"/>
+    <hyperlink ref="G22" r:id="rId19"/>
+    <hyperlink ref="G23" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId12"/>
+  <pageSetup orientation="portrait" r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Formatting done in local supplier section.
</commit_message>
<xml_diff>
--- a/Soldering Tools Required.xlsx
+++ b/Soldering Tools Required.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XPENDER\Documents\GitHub\Electronics-DemandSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -537,7 +537,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -622,12 +622,6 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -648,6 +642,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -981,32 +978,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
+      <c r="A2" s="34"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
@@ -1395,32 +1392,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
+      <c r="A2" s="36"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1753,7 +1750,9 @@
       <c r="K12" s="9"/>
     </row>
     <row r="13" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
+      <c r="A13" s="9">
+        <v>10</v>
+      </c>
       <c r="B13" s="9" t="s">
         <v>70</v>
       </c>
@@ -1787,7 +1786,7 @@
     </row>
     <row r="14" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>69</v>
@@ -1819,219 +1818,242 @@
       <c r="K14" s="9"/>
     </row>
     <row r="15" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="30">
-        <v>11</v>
-      </c>
-      <c r="B15" s="30" t="s">
+      <c r="A15" s="9">
+        <v>12</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="30"/>
+      <c r="I15" s="31">
+        <v>800</v>
+      </c>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+    </row>
+    <row r="16" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="9">
+        <v>13</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" s="9"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="30"/>
+      <c r="I16" s="31">
+        <v>500</v>
+      </c>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+    </row>
+    <row r="17" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9">
+        <v>14</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="9"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="30"/>
+      <c r="I17" s="31">
+        <v>800</v>
+      </c>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="18" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="9">
+        <v>15</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" s="30"/>
+      <c r="I18" s="31">
+        <v>500</v>
+      </c>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+    </row>
+    <row r="19" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9">
+        <v>16</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C19" s="9"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" s="30"/>
+      <c r="I19" s="31">
+        <v>36000</v>
+      </c>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="9">
+        <v>17</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C20" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="31"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="32" t="s">
+      <c r="D20" s="16"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="30" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="32"/>
-      <c r="I15" s="33">
+      <c r="H20" s="30"/>
+      <c r="I20" s="31">
         <v>50000</v>
       </c>
-      <c r="J15" s="30"/>
-      <c r="K15" s="30" t="s">
+      <c r="J20" s="9"/>
+      <c r="K20" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="30"/>
-      <c r="B16" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="32" t="s">
+    <row r="21" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="9">
+        <v>18</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="9"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="H16" s="32"/>
-      <c r="I16" s="33">
-        <v>800</v>
-      </c>
-      <c r="J16" s="30"/>
-      <c r="K16" s="30"/>
-    </row>
-    <row r="17" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="30"/>
-      <c r="B17" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="30"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="32" t="s">
+      <c r="H21" s="30">
+        <v>2</v>
+      </c>
+      <c r="I21" s="31">
+        <v>19500</v>
+      </c>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+    </row>
+    <row r="22" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9">
+        <v>19</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="9"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="H17" s="32"/>
-      <c r="I17" s="33">
-        <v>500</v>
-      </c>
-      <c r="J17" s="30"/>
-      <c r="K17" s="30"/>
-    </row>
-    <row r="18" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="30"/>
-      <c r="B18" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="C18" s="30"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="32" t="s">
+      <c r="H22" s="30">
+        <v>1</v>
+      </c>
+      <c r="I22" s="31">
+        <v>31000</v>
+      </c>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="9">
+        <v>20</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" s="9"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="H18" s="32"/>
-      <c r="I18" s="33">
-        <v>800</v>
-      </c>
-      <c r="J18" s="30"/>
-      <c r="K18" s="30"/>
-    </row>
-    <row r="19" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="30"/>
-      <c r="B19" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="C19" s="30"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="H19" s="32"/>
-      <c r="I19" s="33">
-        <v>500</v>
-      </c>
-      <c r="J19" s="30"/>
-      <c r="K19" s="30"/>
-    </row>
-    <row r="20" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="30"/>
-      <c r="B20" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="H20" s="32"/>
-      <c r="I20" s="33">
-        <v>36000</v>
-      </c>
-      <c r="J20" s="30"/>
-      <c r="K20" s="30" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="30"/>
-      <c r="B21" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="C21" s="30"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="H21" s="32">
+      <c r="H23" s="30">
+        <v>1</v>
+      </c>
+      <c r="I23" s="31">
+        <v>20500</v>
+      </c>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+    </row>
+    <row r="24" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9">
+        <v>21</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" s="9"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="H24" s="30">
         <v>2</v>
       </c>
-      <c r="I21" s="33">
-        <v>19500</v>
-      </c>
-      <c r="J21" s="30"/>
-      <c r="K21" s="30"/>
-    </row>
-    <row r="22" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="30"/>
-      <c r="B22" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="31"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="H22" s="32">
-        <v>1</v>
-      </c>
-      <c r="I22" s="33">
-        <v>31000</v>
-      </c>
-      <c r="J22" s="30"/>
-      <c r="K22" s="30" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="30"/>
-      <c r="B23" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="C23" s="30"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="H23" s="32">
-        <v>1</v>
-      </c>
-      <c r="I23" s="33">
-        <v>20500</v>
-      </c>
-      <c r="J23" s="30"/>
-      <c r="K23" s="30"/>
-    </row>
-    <row r="24" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="30"/>
-      <c r="B24" s="30" t="s">
-        <v>98</v>
-      </c>
-      <c r="C24" s="30"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="H24" s="32">
-        <v>2</v>
-      </c>
-      <c r="I24" s="33">
+      <c r="I24" s="31">
         <v>40000</v>
       </c>
-      <c r="J24" s="30"/>
-      <c r="K24" s="30" t="s">
+      <c r="J24" s="9"/>
+      <c r="K24" s="9" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="17" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
+      <c r="A25" s="9">
+        <v>22</v>
+      </c>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
       <c r="G25" s="28" t="s">
         <v>66</v>
       </c>
@@ -2040,8 +2062,8 @@
         <f>SUM(I4:I24)</f>
         <v>217966</v>
       </c>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I26" s="8"/>
@@ -2146,12 +2168,12 @@
     <hyperlink ref="G11" r:id="rId9"/>
     <hyperlink ref="G12" r:id="rId10"/>
     <hyperlink ref="G14" r:id="rId11"/>
-    <hyperlink ref="G15" r:id="rId12"/>
-    <hyperlink ref="G16" r:id="rId13"/>
-    <hyperlink ref="G17" r:id="rId14"/>
-    <hyperlink ref="G18" r:id="rId15"/>
-    <hyperlink ref="G19" r:id="rId16"/>
-    <hyperlink ref="G20" r:id="rId17"/>
+    <hyperlink ref="G20" r:id="rId12"/>
+    <hyperlink ref="G15" r:id="rId13"/>
+    <hyperlink ref="G16" r:id="rId14"/>
+    <hyperlink ref="G17" r:id="rId15"/>
+    <hyperlink ref="G18" r:id="rId16"/>
+    <hyperlink ref="G19" r:id="rId17"/>
     <hyperlink ref="G21" r:id="rId18"/>
     <hyperlink ref="G22" r:id="rId19"/>
     <hyperlink ref="G23" r:id="rId20"/>

</xml_diff>